<commit_message>
Expand v5 helper section: granular wage/BI/CG breakouts + named ranges
Helper / Tax-Calc Inputs section now splits each major category for
LAMBDA consumption:
- Wages: W2_OWNER (S-Corp reasonable comp) | W2_THIRD_PARTY | W2_TOTAL
- Business Income: BI_SE_SUBJECT (Sch C/F + active K-1 PTP) |
  BI_ACTIVE_NONSE (active S-Corp K-1, etc.) | BI_PASSIVE (passive K-1s,
  Sch E rental)
- Investment carve-outs: TAX_EXEMPT, QUAL_DIV
- Capital Gains: CG_LT, CG_ST (Sch D nets to Line 7 but LAMBDAs need
  them split for ordinary vs preferential rate), SEC1250 sub-carve

Each helper label is a workbook-level named range pointing at its
amount cell, so future LAMBDAs / summary page can reference as
=W2_OWNER, =BI_SE_SUBJECT, etc. directly. Key rollup totals also
named: TotalIncome, AGI, StdItemDed, QBI_Deduction, TaxableIncome,
plus per-line Effective values (Line_1z_Wages, Line_7_CapGain, ...).
</commit_message>
<xml_diff>
--- a/docs/Tax_Workbook_Sample_Template_v5.xlsx
+++ b/docs/Tax_Workbook_Sample_Template_v5.xlsx
@@ -35,6 +35,28 @@
     <definedName name="Itemized_Docs">'Dropdown_Lists'!$F$35:$F$38</definedName>
     <definedName name="Credit_Docs">'Dropdown_Lists'!$G$35:$G$37</definedName>
     <definedName name="Payment_Docs">'Dropdown_Lists'!$H$35:$H$36</definedName>
+    <definedName name="W2_OWNER">'Y2025'!$J$21</definedName>
+    <definedName name="W2_THIRD_PARTY">'Y2025'!$J$22</definedName>
+    <definedName name="W2_TOTAL">'Y2025'!$J$23</definedName>
+    <definedName name="BI_SE_SUBJECT">'Y2025'!$J$24</definedName>
+    <definedName name="BI_ACTIVE_NONSE">'Y2025'!$J$25</definedName>
+    <definedName name="BI_PASSIVE">'Y2025'!$J$26</definedName>
+    <definedName name="TAX_EXEMPT">'Y2025'!$J$27</definedName>
+    <definedName name="QUAL_DIV">'Y2025'!$J$28</definedName>
+    <definedName name="CG_LT">'Y2025'!$J$29</definedName>
+    <definedName name="CG_ST">'Y2025'!$J$30</definedName>
+    <definedName name="SEC1250">'Y2025'!$J$31</definedName>
+    <definedName name="Line_1z_Wages">'Y2025'!$M$6</definedName>
+    <definedName name="Line_2b_TaxInt">'Y2025'!$M$7</definedName>
+    <definedName name="Line_3b_OrdDiv">'Y2025'!$M$8</definedName>
+    <definedName name="Line_7_CapGain">'Y2025'!$M$9</definedName>
+    <definedName name="Line_8_OtherInc">'Y2025'!$M$10</definedName>
+    <definedName name="TotalIncome">'Y2025'!$M$11</definedName>
+    <definedName name="AdjToIncome">'Y2025'!$M$12</definedName>
+    <definedName name="AGI">'Y2025'!$M$13</definedName>
+    <definedName name="StdItemDed">'Y2025'!$M$14</definedName>
+    <definedName name="QBI_Deduction">'Y2025'!$M$15</definedName>
+    <definedName name="TaxableIncome">'Y2025'!$M$16</definedName>
     <definedName name="Drill_Line">'Y2025'!$I$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2151,147 +2173,231 @@
     <row r="21">
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>TAX_EXEMPT</t>
+          <t>W2_OWNER</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Tax-exempt interest (Line 2a; reported but not taxed)</t>
+          <t>Owner W-2 wages (S-Corp reasonable comp; Treatment_Profile=W2_SCorpOwner)</t>
         </is>
       </c>
       <c r="J21">
-        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "TAX_EXEMPT")</f>
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "W2_SCorpOwner")</f>
         <v/>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>NIIT_FN (MAGI base)</t>
+          <t>FICA_Employer/Employee — True Tax Burden box</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>QUAL_DIV</t>
+          <t>W2_THIRD_PARTY</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Qualified dividends (carve-out of Line 3b; LTCG stack)</t>
+          <t>Third-party W-2 wages (Treatment_Profile=W2_Employee)</t>
         </is>
       </c>
       <c r="J22">
-        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "QUAL_DIV")</f>
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "W2_Employee")</f>
         <v/>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Calc_CapGainsTax stacking</t>
+          <t>Calc_SE_Tax (SS-base sharing) · AddlMedicareTax_FN</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>OWNER_PAY</t>
+          <t>W2_TOTAL</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Owner W-2 wages (S-Corp reasonable comp)</t>
+          <t>Total W-2 wages (owner + third-party)</t>
         </is>
       </c>
       <c r="J23">
-        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "OWNER_PAY")</f>
+        <f>W2_OWNER+W2_THIRD_PARTY</f>
         <v/>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>FICA_Employer/Employee — True Tax Burden box</t>
+          <t>Calc_SE_Tax (SS-base sharing) · AddlMedicareTax_FN</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>SEC1250</t>
+          <t>BI_SE_SUBJECT</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>§1250 unrecaptured gain (capped at 25% rate)</t>
+          <t>Business income subject to SE tax (Sch C, Sch F, active K-1 PTP)</t>
         </is>
       </c>
       <c r="J24">
-        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "SEC1250")</f>
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Bucket], "Business Income", tblMaster_Inputs[SE_Subject], "Yes")</f>
         <v/>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Calc_1250Tax</t>
+          <t>Calc_SE_Tax base · AddlMedicareTax_FN</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>SE_INCOME</t>
+          <t>BI_ACTIVE_NONSE</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Total SE-subject income (Sch C/F + active K-1 helper)</t>
+          <t>Active business income NOT subject to SE (active S-Corp K-1, etc.)</t>
         </is>
       </c>
       <c r="J25">
-        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "SE_INCOME") + SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "SchC_Active") + SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "SchF_Active")</f>
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Bucket], "Business Income", tblMaster_Inputs[SE_Subject], "No", tblMaster_Inputs[NIIT_Class], "Active")</f>
         <v/>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Calc_SE_Tax · AddlMedicareTax_FN</t>
+          <t>NIIT exclusion (active) · QBI eligible</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>PASSIVE</t>
+          <t>BI_PASSIVE</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Passive income/loss (Sch E baseline; PAL limits)</t>
+          <t>Passive business income / loss (passive K-1s, Sch E rental)</t>
         </is>
       </c>
       <c r="J26">
-        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[NIIT_Class], "Passive")</f>
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Bucket], "Business Income", tblMaster_Inputs[NIIT_Class], "Passive")</f>
         <v/>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>PassiveLossAllowed_FN</t>
+          <t>PassiveLossAllowed_FN · NIIT inclusion</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>TAX_W2</t>
+          <t>TAX_EXEMPT</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Total W-2 wages (any source)</t>
+          <t>Tax-exempt interest (Line 2a; reported but not taxed)</t>
         </is>
       </c>
       <c r="J27">
-        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Bucket], "Wages")</f>
+        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "TAX_EXEMPT")</f>
         <v/>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Calc_SE_Tax · AddlMedicareTax_FN</t>
+          <t>NIIT_FN (MAGI base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>QUAL_DIV</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Qualified dividends (carve-out of Line 3b; LTCG stack)</t>
+        </is>
+      </c>
+      <c r="J28">
+        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "QUAL_DIV")</f>
+        <v/>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Calc_CapGainsTax stacking</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>CG_LT</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Long-term capital gains (LT preferential rate; stacks with qualified div)</t>
+        </is>
+      </c>
+      <c r="J29">
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "LTCG_Stock") + SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "LTCG_RE") + SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "LTCG_K1_Passthrough") + SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "Sec1250_Recap")</f>
+        <v/>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Calc_CapGainsTax</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>CG_ST</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Short-term capital gains (taxed as ordinary income)</t>
+        </is>
+      </c>
+      <c r="J30">
+        <f>SUMIFS(tblMaster_Inputs[Baseline_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Treatment_Profile], "STCG_Stock")</f>
+        <v/>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Calc_OrdinaryTax (ST folded into ordinary income)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>SEC1250</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>§1250 unrecaptured gain (sub-carve of CG_LT; capped at 25% rate)</t>
+        </is>
+      </c>
+      <c r="J31">
+        <f>SUMIFS(tblMaster_Inputs[Helper_Amount], tblMaster_Inputs[Year], 2025, tblMaster_Inputs[Helper_Treatment], "SEC1250")</f>
+        <v/>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Calc_1250Tax</t>
         </is>
       </c>
     </row>

</xml_diff>